<commit_message>
Se corrigio error excel
</commit_message>
<xml_diff>
--- a/ProyectoAsistencia/ReporteEquiposLaboratorio.xlsx
+++ b/ProyectoAsistencia/ReporteEquiposLaboratorio.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="46">
   <si>
     <t>Nro Laboratorio</t>
   </si>
@@ -32,34 +32,124 @@
     <t>1</t>
   </si>
   <si>
+    <t>Teclado</t>
+  </si>
+  <si>
+    <t>EQ001</t>
+  </si>
+  <si>
+    <t>SN1234567890</t>
+  </si>
+  <si>
+    <t>OPERATIVO</t>
+  </si>
+  <si>
     <t>CPU</t>
   </si>
   <si>
-    <t>123</t>
-  </si>
-  <si>
-    <t>Operativo</t>
+    <t>EQ002</t>
+  </si>
+  <si>
+    <t>SN9876543210</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
+    <t>PizarraDigital</t>
+  </si>
+  <si>
+    <t>EQ004</t>
+  </si>
+  <si>
+    <t>SN2233445566</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>EQ006</t>
+  </si>
+  <si>
+    <t>SN4455667788</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>Monitor</t>
   </si>
   <si>
-    <t>1232133212</t>
-  </si>
-  <si>
-    <t>123123</t>
-  </si>
-  <si>
-    <t>Teclado</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>12</t>
+    <t>EQ007</t>
+  </si>
+  <si>
+    <t>SN5566778899</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>EQ009</t>
+  </si>
+  <si>
+    <t>SN7788990011</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>EQ011</t>
+  </si>
+  <si>
+    <t>SN9900112233</t>
+  </si>
+  <si>
+    <t>EQ013</t>
+  </si>
+  <si>
+    <t>SN1122334455</t>
+  </si>
+  <si>
+    <t>EQ015</t>
+  </si>
+  <si>
+    <t>SN3344556677</t>
+  </si>
+  <si>
+    <t>EQ017</t>
+  </si>
+  <si>
+    <t>EQ019</t>
+  </si>
+  <si>
+    <t>EQ021</t>
+  </si>
+  <si>
+    <t>EQ023</t>
+  </si>
+  <si>
+    <t>EQ025</t>
+  </si>
+  <si>
+    <t>EQ027</t>
+  </si>
+  <si>
+    <t>EQ029</t>
+  </si>
+  <si>
+    <t>EQ031</t>
+  </si>
+  <si>
+    <t>EQ033</t>
+  </si>
+  <si>
+    <t>EQ035</t>
+  </si>
+  <si>
+    <t>EQ037</t>
+  </si>
+  <si>
+    <t>EQ039</t>
   </si>
 </sst>
 </file>
@@ -104,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.0" customWidth="true"/>
@@ -142,15 +232,15 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -162,41 +252,330 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>